<commit_message>
cron: phases A, B finished
</commit_message>
<xml_diff>
--- a/test-docs/collections/cron/cron.xlsx
+++ b/test-docs/collections/cron/cron.xlsx
@@ -11,7 +11,7 @@
     <sheet name="COL-cron" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COL-cron'!$A$4:$F$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COL-cron'!$A$4:$F$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1443,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1463,7 +1463,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>COL-cron — Curated Test Collection (active; 68 TCs referenced; vacation s135 + reports s136 + cross-service s137)</t>
+          <t>COL-cron — Curated Test Collection (complete; 87 TCs referenced; vacation s135 + reports s136 + cross-service s137 + statistics + email s138)</t>
         </is>
       </c>
     </row>
@@ -3675,8 +3675,616 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>TC-STAT-077</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>StatisticReportScheduler — cron fires at 04:00 NSK, ShedLock acquired/released, start/finish markers emit</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr">
+        <is>
+          <t>Row 22 happy-path; baseline periodic sync with ShedLock</t>
+        </is>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>TC-STAT-078</t>
+        </is>
+      </c>
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Delta #8 regression — statistic-report sync failure logged at INFO (level:6), NOT ERROR (level:3)</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
+        <is>
+          <t>Row 22 design issue; delta #8 log-level regression guard</t>
+        </is>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>TC-STAT-079</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>#3345 Bug 1 regression — employment-period filter excludes pre-hire and post-leave months</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>Row 22 regression; #3345 MR !5101 fix</t>
+        </is>
+      </c>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>TC-STAT-080</t>
+        </is>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>#3345 Bug 2 regression — day-off reschedule triggers month_norm recalc via RabbitMQ event</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Row 22 regression; #3345 event-fan-out fix</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="15" t="inlineStr">
+        <is>
+          <t>TC-STAT-081</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C77" s="15" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
+          <t>#3337 regression — sick-leave creation updates month_norm and reported_effort via SICK_LEAVE_CHANGES event</t>
+        </is>
+      </c>
+      <c r="E77" s="15" t="inlineStr">
+        <is>
+          <t>Row 22 regression; #3337 event-enum broadening</t>
+        </is>
+      </c>
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>TC-STAT-082</t>
+        </is>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>#3337 regression — scoped event for employee A does NOT delete statistic_report rows for employee B</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>Row 22 regression; #3337 scoped-delete fix</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="15" t="inlineStr">
+        <is>
+          <t>TC-STAT-083</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C79" s="15" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>#3346 regression (bug #895498) — manual statistic_report row delete is restored on next optimized sync</t>
+        </is>
+      </c>
+      <c r="E79" s="15" t="inlineStr">
+        <is>
+          <t>Row 22 regression; #3346 scheduler-wiring fix</t>
+        </is>
+      </c>
+      <c r="F79" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>TC-STAT-084</t>
+        </is>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>statistics</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>TS-Stat-CronStatReportSync</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Full vs optimized sync contract — full refreshes previous + current year; optimized refreshes previous + current month only</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Row 22 endpoint-contract; #3345 note 894873</t>
+        </is>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-001</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>EmailSendScheduler — cron fires every 20 s, ShedLock acquired/released, start/finish markers emit</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>Row 8 happy-path; baseline dispatcher cadence + lock</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-002</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>Dispatch — NEW email transitions to SENT after SMTP success (happy path)</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>Row 8 SMTP-success status transition</t>
+        </is>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-003</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C83" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>Dispatch — invalid recipient transitions NEW → INVALID (SendFailedException path)</t>
+        </is>
+      </c>
+      <c r="E83" s="15" t="inlineStr">
+        <is>
+          <t>Row 8 invalid-recipient status transition</t>
+        </is>
+      </c>
+      <c r="F83" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-004</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr">
+        <is>
+          <t>Dispatch — partial SMTP failure sets FAILED for rejected messages, SENT for accepted</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>Row 8 mixed-batch status transitions; DI-EMAIL-DISPATCH-RETRY context</t>
+        </is>
+      </c>
+      <c r="F84" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-005</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>DI-EMAIL-DISPATCH-AUTH regression — MailAuthenticationException caught, status NOT updated, infinite retry loop</t>
+        </is>
+      </c>
+      <c r="E85" s="15" t="inlineStr">
+        <is>
+          <t>Row 8 design-issue regression guard; stuck-as-NEW infinite loop</t>
+        </is>
+      </c>
+      <c r="F85" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="16" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-006</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>TS-Email-CronDispatch</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>Dispatch — pageSize = 300 caps per-batch dispatch; overflow drains in subsequent ticks</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>Row 8 batch-size contract; pagination window</t>
+        </is>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-007</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C87" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronPrune</t>
+        </is>
+      </c>
+      <c r="D87" s="15" t="inlineStr">
+        <is>
+          <t>EmailPruneScheduler — cron fires daily at 00:00, ShedLock acquired/released, start/finish markers emit</t>
+        </is>
+      </c>
+      <c r="E87" s="15" t="inlineStr">
+        <is>
+          <t>Row 9 happy-path; baseline retention scheduler</t>
+        </is>
+      </c>
+      <c r="F87" s="15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="16" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-008</t>
+        </is>
+      </c>
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="inlineStr">
+        <is>
+          <t>TS-Email-CronPrune</t>
+        </is>
+      </c>
+      <c r="D88" s="16" t="inlineStr">
+        <is>
+          <t>Retention — emails older than 30 days deleted, emails newer than 30 days preserved</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>Row 9 retention baseline; PT30D cutoff</t>
+        </is>
+      </c>
+      <c r="F88" s="16" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-009</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C89" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronPrune</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>Retention boundary — email exactly at 30-day cutoff behavior (strict less-than: &lt;30d preserved, =30d deleted)</t>
+        </is>
+      </c>
+      <c r="E89" s="15" t="inlineStr">
+        <is>
+          <t>Row 9 off-by-one guard on strict less-than ADD_TIME.lessThan</t>
+        </is>
+      </c>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-010</t>
+        </is>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>TS-Email-CronPrune</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>Retention — attachments deleted with parent email (no FK orphans)</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>Row 9 cascade-delete contract; zero orphans</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="15" t="inlineStr">
+        <is>
+          <t>TC-EMAIL-011</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C91" s="15" t="inlineStr">
+        <is>
+          <t>TS-Email-CronPrune</t>
+        </is>
+      </c>
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>Retention no-op — all emails within retention window; finish marker reports 0 deleted</t>
+        </is>
+      </c>
+      <c r="E91" s="15" t="inlineStr">
+        <is>
+          <t>Row 9 no-op idempotency; zero-delete path</t>
+        </is>
+      </c>
+      <c r="F91" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F72"/>
+  <autoFilter ref="A4:F91"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A5:F5"/>

</xml_diff>